<commit_message>
feat: enhance AnexoPublicaciones report with detailed publication counts and update related Excel template
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Dashboard_v2/src/Infrastructure/Templates/AnexoPublicaciones.xlsx
+++ b/Dashboard_v2/src/Infrastructure/Templates/AnexoPublicaciones.xlsx
@@ -77,6 +77,27 @@
   </x:si>
   <x:si>
     <x:t>Cantidad de ponencias de eventos nacionales e internacionales publicadas con ISSN o ISBN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{G1Count}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{G2Count}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{G3Count}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{G4Count}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{CapitulosCount}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{LibrosMonografiasCount}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{ArticulosDivulgacionCount}}</x:t>
   </x:si>
   <x:si>
     <x:t>No</x:t>
@@ -261,7 +282,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -276,6 +297,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -616,7 +641,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
+      <x:c r="C2" s="4" t="s">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="D2" s="3"/>
     </x:row>
     <x:row r="3" spans="1:4">
@@ -624,7 +651,9 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
+      <x:c r="C3" s="4" t="s">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="D3" s="3"/>
     </x:row>
     <x:row r="4" spans="1:4">
@@ -632,7 +661,9 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
-      <x:c r="C4" s="3"/>
+      <x:c r="C4" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="D4" s="3"/>
     </x:row>
     <x:row r="5" spans="1:4">
@@ -640,7 +671,9 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B5" s="3"/>
-      <x:c r="C5" s="3"/>
+      <x:c r="C5" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="D5" s="3"/>
     </x:row>
     <x:row r="6" spans="1:4">
@@ -648,7 +681,9 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
+      <x:c r="C6" s="4" t="s">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="D6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:4">
@@ -656,7 +691,9 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B7" s="3"/>
-      <x:c r="C7" s="3"/>
+      <x:c r="C7" s="4" t="s">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="D7" s="3"/>
     </x:row>
     <x:row r="8" spans="1:4">
@@ -680,7 +717,9 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B10" s="3"/>
-      <x:c r="C10" s="3"/>
+      <x:c r="C10" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" spans="1:4" ht="32.25" customHeight="1">
@@ -734,62 +773,62 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
-      <x:c r="A2" s="4" t="s">
-        <x:v>22</x:v>
+      <x:c r="A2" s="5" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -818,53 +857,53 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
-      <x:c r="A2" s="4" t="s">
-        <x:v>22</x:v>
+      <x:c r="A2" s="5" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -893,53 +932,53 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
-      <x:c r="A2" s="4" t="s">
-        <x:v>22</x:v>
+      <x:c r="A2" s="5" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -968,53 +1007,53 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
-      <x:c r="A2" s="4" t="s">
-        <x:v>22</x:v>
+      <x:c r="A2" s="5" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1042,183 +1081,183 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:5">
-      <x:c r="A1" s="5" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B1" s="6"/>
-      <x:c r="C1" s="6"/>
-      <x:c r="D1" s="6"/>
-      <x:c r="E1" s="7"/>
+      <x:c r="A1" s="6" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B1" s="7"/>
+      <x:c r="C1" s="7"/>
+      <x:c r="D1" s="7"/>
+      <x:c r="E1" s="8"/>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="5" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
+      <x:c r="D3" s="2" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5">
-      <x:c r="A3" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
-      <x:c r="A6" s="5" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B6" s="6"/>
-      <x:c r="C6" s="6"/>
-      <x:c r="D6" s="6"/>
-      <x:c r="E6" s="7"/>
+      <x:c r="A6" s="6" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="7"/>
+      <x:c r="E6" s="8"/>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:5">
+      <x:c r="A8" s="5" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
+      <x:c r="D8" s="2" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:5">
-      <x:c r="A8" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C8" s="2" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D8" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E8" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:5">
-      <x:c r="A11" s="5" t="s">
+      <x:c r="A11" s="6" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B11" s="6"/>
-      <x:c r="C11" s="6"/>
-      <x:c r="D11" s="6"/>
-      <x:c r="E11" s="7"/>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="7"/>
+      <x:c r="E11" s="8"/>
     </x:row>
     <x:row r="12" spans="1:5">
       <x:c r="A12" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E12" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:5">
+      <x:c r="A13" s="5" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
+      <x:c r="D13" s="2" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="E12" s="1" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:5">
-      <x:c r="A13" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B13" s="2" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C13" s="2" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D13" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E13" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:5">
       <x:c r="A14" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1252,62 +1291,62 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
-      <x:c r="A2" s="4" t="s">
-        <x:v>22</x:v>
+      <x:c r="A2" s="5" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>